<commit_message>
actualizacion catalogo de productos
</commit_message>
<xml_diff>
--- a/data/SKU_BX.xlsx
+++ b/data/SKU_BX.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ccusi\Documents\Proyect_Coder\G360-ecosystem\projects\g360-master-data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F35675C5-EC64-4E91-B2C6-7745B518458B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE3D6777-B383-4A46-9E39-436827E4A01D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6630" yWindow="750" windowWidth="14565" windowHeight="11550" xr2:uid="{B19518BF-BEE8-4C61-8490-6B34AC0E6445}"/>
+    <workbookView xWindow="6165" yWindow="2160" windowWidth="20865" windowHeight="11565" xr2:uid="{B19518BF-BEE8-4C61-8490-6B34AC0E6445}"/>
   </bookViews>
   <sheets>
     <sheet name="SKU_BX" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2238" uniqueCount="1024">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2038" uniqueCount="1025">
   <si>
     <t>85609</t>
   </si>
@@ -2949,9 +2949,6 @@
     <t>TRADICIONAL</t>
   </si>
   <si>
-    <t>016728</t>
-  </si>
-  <si>
     <t>011372</t>
   </si>
   <si>
@@ -3106,6 +3103,12 @@
   </si>
   <si>
     <t>78532</t>
+  </si>
+  <si>
+    <t>MA014</t>
+  </si>
+  <si>
+    <t>016788</t>
   </si>
 </sst>
 </file>
@@ -3201,10 +3204,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2A1D9BEB-E717-47EE-8455-B1311A6622FA}" name="Tabla2" displayName="Tabla2" ref="A1:D1118" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:D1118" xr:uid="{34683EFA-A54F-4EC3-B9AE-5709FCB52753}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D1118">
-    <sortCondition ref="A1:A1118"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{2A1D9BEB-E717-47EE-8455-B1311A6622FA}" name="Tabla2" displayName="Tabla2" ref="A1:D1018" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:D1018" xr:uid="{34683EFA-A54F-4EC3-B9AE-5709FCB52753}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D1018">
+    <sortCondition ref="A1:A1119"/>
   </sortState>
   <tableColumns count="4">
     <tableColumn id="1" xr3:uid="{EC5719B2-2D0A-4AF8-AAD3-3D55FB38D389}" name="ORDEN"/>
@@ -3501,7 +3504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{555D8C85-EBC5-428E-83BD-D5EBEE488AE6}">
-  <dimension ref="A1:D1118"/>
+  <dimension ref="A1:D1018"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8.42578125" customWidth="1"/>
@@ -3892,8 +3895,8 @@
       <c r="A28">
         <v>27</v>
       </c>
-      <c r="B28" t="s">
-        <v>971</v>
+      <c r="B28" s="1" t="s">
+        <v>1024</v>
       </c>
       <c r="C28">
         <v>50</v>
@@ -6609,7 +6612,7 @@
         <v>221</v>
       </c>
       <c r="B222" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="C222">
         <v>36</v>
@@ -6623,7 +6626,7 @@
         <v>222</v>
       </c>
       <c r="B223" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="C223">
         <v>36</v>
@@ -6637,7 +6640,7 @@
         <v>223</v>
       </c>
       <c r="B224" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="C224">
         <v>36</v>
@@ -6665,7 +6668,7 @@
         <v>225</v>
       </c>
       <c r="B226" t="s">
-        <v>975</v>
+        <v>974</v>
       </c>
       <c r="C226">
         <v>25</v>
@@ -6707,7 +6710,7 @@
         <v>228</v>
       </c>
       <c r="B229" t="s">
-        <v>976</v>
+        <v>975</v>
       </c>
       <c r="C229">
         <v>50</v>
@@ -6791,7 +6794,7 @@
         <v>234</v>
       </c>
       <c r="B235" t="s">
-        <v>977</v>
+        <v>976</v>
       </c>
       <c r="C235">
         <v>18</v>
@@ -6819,7 +6822,7 @@
         <v>236</v>
       </c>
       <c r="B237" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="C237">
         <v>36</v>
@@ -7449,7 +7452,7 @@
         <v>281</v>
       </c>
       <c r="B282" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="C282">
         <v>100</v>
@@ -7967,7 +7970,7 @@
         <v>318</v>
       </c>
       <c r="B319" t="s">
-        <v>980</v>
+        <v>979</v>
       </c>
       <c r="C319">
         <v>100</v>
@@ -7981,7 +7984,7 @@
         <v>319</v>
       </c>
       <c r="B320" t="s">
-        <v>981</v>
+        <v>980</v>
       </c>
       <c r="C320">
         <v>100</v>
@@ -7995,7 +7998,7 @@
         <v>320</v>
       </c>
       <c r="B321" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="C321">
         <v>100</v>
@@ -8009,7 +8012,7 @@
         <v>321</v>
       </c>
       <c r="B322" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="C322">
         <v>100</v>
@@ -8023,7 +8026,7 @@
         <v>322</v>
       </c>
       <c r="B323" t="s">
-        <v>984</v>
+        <v>983</v>
       </c>
       <c r="C323">
         <v>100</v>
@@ -8135,7 +8138,7 @@
         <v>330</v>
       </c>
       <c r="B331" t="s">
-        <v>985</v>
+        <v>984</v>
       </c>
       <c r="C331">
         <v>100</v>
@@ -8149,7 +8152,7 @@
         <v>331</v>
       </c>
       <c r="B332" t="s">
-        <v>986</v>
+        <v>985</v>
       </c>
       <c r="C332">
         <v>100</v>
@@ -8163,7 +8166,7 @@
         <v>332</v>
       </c>
       <c r="B333" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="C333">
         <v>100</v>
@@ -8177,7 +8180,7 @@
         <v>333</v>
       </c>
       <c r="B334" t="s">
-        <v>988</v>
+        <v>987</v>
       </c>
       <c r="C334">
         <v>100</v>
@@ -8191,7 +8194,7 @@
         <v>334</v>
       </c>
       <c r="B335" t="s">
-        <v>989</v>
+        <v>988</v>
       </c>
       <c r="C335">
         <v>100</v>
@@ -8275,7 +8278,7 @@
         <v>340</v>
       </c>
       <c r="B341" t="s">
-        <v>990</v>
+        <v>989</v>
       </c>
       <c r="C341">
         <v>120</v>
@@ -8485,7 +8488,7 @@
         <v>355</v>
       </c>
       <c r="B356" t="s">
-        <v>991</v>
+        <v>990</v>
       </c>
       <c r="C356">
         <v>24</v>
@@ -9185,7 +9188,7 @@
         <v>405</v>
       </c>
       <c r="B406" t="s">
-        <v>992</v>
+        <v>991</v>
       </c>
       <c r="C406">
         <v>576</v>
@@ -10067,7 +10070,7 @@
         <v>468</v>
       </c>
       <c r="B469" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="C469">
         <v>432</v>
@@ -10081,7 +10084,7 @@
         <v>469</v>
       </c>
       <c r="B470" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C470">
         <v>432</v>
@@ -10095,7 +10098,7 @@
         <v>470</v>
       </c>
       <c r="B471" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="C471">
         <v>432</v>
@@ -10109,7 +10112,7 @@
         <v>471</v>
       </c>
       <c r="B472" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="C472">
         <v>36</v>
@@ -10123,7 +10126,7 @@
         <v>472</v>
       </c>
       <c r="B473" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="C473">
         <v>36</v>
@@ -10137,7 +10140,7 @@
         <v>473</v>
       </c>
       <c r="B474" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="C474">
         <v>36</v>
@@ -10193,7 +10196,7 @@
         <v>477</v>
       </c>
       <c r="B478" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="C478">
         <v>1152</v>
@@ -10361,7 +10364,7 @@
         <v>489</v>
       </c>
       <c r="B490" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="C490">
         <v>864</v>
@@ -10375,7 +10378,7 @@
         <v>490</v>
       </c>
       <c r="B491" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="C491">
         <v>864</v>
@@ -10389,7 +10392,7 @@
         <v>491</v>
       </c>
       <c r="B492" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="C492">
         <v>864</v>
@@ -10403,7 +10406,7 @@
         <v>492</v>
       </c>
       <c r="B493" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="C493">
         <v>864</v>
@@ -11565,7 +11568,7 @@
         <v>575</v>
       </c>
       <c r="B576" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="C576">
         <v>144</v>
@@ -11579,7 +11582,7 @@
         <v>576</v>
       </c>
       <c r="B577" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="C577">
         <v>96</v>
@@ -11593,7 +11596,7 @@
         <v>577</v>
       </c>
       <c r="B578" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="C578">
         <v>96</v>
@@ -11607,7 +11610,7 @@
         <v>578</v>
       </c>
       <c r="B579" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="C579">
         <v>96</v>
@@ -11635,7 +11638,7 @@
         <v>580</v>
       </c>
       <c r="B581" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="C581">
         <v>48</v>
@@ -11649,7 +11652,7 @@
         <v>581</v>
       </c>
       <c r="B582" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="C582">
         <v>576</v>
@@ -11663,7 +11666,7 @@
         <v>582</v>
       </c>
       <c r="B583" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="C583">
         <v>576</v>
@@ -11677,7 +11680,7 @@
         <v>583</v>
       </c>
       <c r="B584" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="C584">
         <v>576</v>
@@ -11691,7 +11694,7 @@
         <v>584</v>
       </c>
       <c r="B585" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="C585">
         <v>576</v>
@@ -11705,7 +11708,7 @@
         <v>585</v>
       </c>
       <c r="B586" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="C586">
         <v>576</v>
@@ -11719,7 +11722,7 @@
         <v>586</v>
       </c>
       <c r="B587" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="C587">
         <v>28</v>
@@ -11817,7 +11820,7 @@
         <v>593</v>
       </c>
       <c r="B594" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="C594">
         <v>576</v>
@@ -11929,7 +11932,7 @@
         <v>601</v>
       </c>
       <c r="B602" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="C602">
         <v>576</v>
@@ -11985,7 +11988,7 @@
         <v>605</v>
       </c>
       <c r="B606" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="C606">
         <v>576</v>
@@ -12139,7 +12142,7 @@
         <v>616</v>
       </c>
       <c r="B617" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="C617">
         <v>576</v>
@@ -12153,7 +12156,7 @@
         <v>617</v>
       </c>
       <c r="B618" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="C618">
         <v>576</v>
@@ -12167,7 +12170,7 @@
         <v>618</v>
       </c>
       <c r="B619" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="C619">
         <v>576</v>
@@ -12965,7 +12968,7 @@
         <v>675</v>
       </c>
       <c r="B676" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="C676">
         <v>100</v>
@@ -14449,7 +14452,7 @@
         <v>781</v>
       </c>
       <c r="B782" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="C782">
         <v>5</v>
@@ -14897,7 +14900,7 @@
         <v>813</v>
       </c>
       <c r="B814" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="C814">
         <v>5</v>
@@ -17749,1417 +17752,14 @@
       </c>
     </row>
     <row r="1018" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1018">
-        <v>1017</v>
-      </c>
       <c r="B1018" t="s">
-        <v>100</v>
+        <v>1023</v>
       </c>
       <c r="C1018">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="D1018" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1019" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1019">
-        <v>1018</v>
-      </c>
-      <c r="B1019" t="s">
-        <v>99</v>
-      </c>
-      <c r="C1019">
-        <v>5</v>
-      </c>
-      <c r="D1019" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1020" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1020">
-        <v>1019</v>
-      </c>
-      <c r="B1020" t="s">
-        <v>98</v>
-      </c>
-      <c r="C1020">
-        <v>5</v>
-      </c>
-      <c r="D1020" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1021" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1021">
-        <v>1020</v>
-      </c>
-      <c r="B1021" t="s">
-        <v>97</v>
-      </c>
-      <c r="C1021">
-        <v>6</v>
-      </c>
-      <c r="D1021" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1022" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1022">
-        <v>1021</v>
-      </c>
-      <c r="B1022" t="s">
-        <v>96</v>
-      </c>
-      <c r="C1022">
-        <v>6</v>
-      </c>
-      <c r="D1022" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1023" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1023">
-        <v>1022</v>
-      </c>
-      <c r="B1023" t="s">
-        <v>95</v>
-      </c>
-      <c r="C1023">
-        <v>6</v>
-      </c>
-      <c r="D1023" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1024" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1024">
-        <v>1023</v>
-      </c>
-      <c r="B1024" t="s">
-        <v>94</v>
-      </c>
-      <c r="C1024">
-        <v>6</v>
-      </c>
-      <c r="D1024" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1025" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1025">
-        <v>1024</v>
-      </c>
-      <c r="B1025" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1025">
-        <v>200</v>
-      </c>
-      <c r="D1025" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1026" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1026">
-        <v>1025</v>
-      </c>
-      <c r="B1026" t="s">
-        <v>92</v>
-      </c>
-      <c r="C1026">
-        <v>56</v>
-      </c>
-      <c r="D1026" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1027" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1027">
-        <v>1026</v>
-      </c>
-      <c r="B1027" t="s">
-        <v>91</v>
-      </c>
-      <c r="C1027">
-        <v>120</v>
-      </c>
-      <c r="D1027" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1028" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1028">
-        <v>1027</v>
-      </c>
-      <c r="B1028" t="s">
-        <v>90</v>
-      </c>
-      <c r="C1028">
-        <v>120</v>
-      </c>
-      <c r="D1028" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1029" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1029">
-        <v>1028</v>
-      </c>
-      <c r="B1029" t="s">
-        <v>89</v>
-      </c>
-      <c r="C1029">
-        <v>18</v>
-      </c>
-      <c r="D1029" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1030" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1030">
-        <v>1029</v>
-      </c>
-      <c r="B1030" t="s">
-        <v>88</v>
-      </c>
-      <c r="C1030">
-        <v>6</v>
-      </c>
-      <c r="D1030" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1031" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1031">
-        <v>1030</v>
-      </c>
-      <c r="B1031" t="s">
-        <v>87</v>
-      </c>
-      <c r="C1031">
-        <v>54</v>
-      </c>
-      <c r="D1031" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1032" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1032">
-        <v>1031</v>
-      </c>
-      <c r="B1032" t="s">
-        <v>86</v>
-      </c>
-      <c r="C1032">
-        <v>10</v>
-      </c>
-      <c r="D1032" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1033" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1033">
-        <v>1032</v>
-      </c>
-      <c r="B1033" t="s">
-        <v>85</v>
-      </c>
-      <c r="C1033">
-        <v>12</v>
-      </c>
-      <c r="D1033" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1034" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1034">
-        <v>1033</v>
-      </c>
-      <c r="B1034" t="s">
-        <v>84</v>
-      </c>
-      <c r="C1034">
-        <v>12</v>
-      </c>
-      <c r="D1034" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1035" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1035">
-        <v>1034</v>
-      </c>
-      <c r="B1035" t="s">
-        <v>83</v>
-      </c>
-      <c r="C1035">
-        <v>5</v>
-      </c>
-      <c r="D1035" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1036" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1036">
-        <v>1035</v>
-      </c>
-      <c r="B1036" t="s">
-        <v>82</v>
-      </c>
-      <c r="C1036">
-        <v>800</v>
-      </c>
-      <c r="D1036" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1037" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1037">
-        <v>1036</v>
-      </c>
-      <c r="B1037" t="s">
-        <v>81</v>
-      </c>
-      <c r="C1037">
-        <v>5</v>
-      </c>
-      <c r="D1037" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1038" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1038">
-        <v>1037</v>
-      </c>
-      <c r="B1038" t="s">
-        <v>80</v>
-      </c>
-      <c r="C1038">
-        <v>5</v>
-      </c>
-      <c r="D1038" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1039" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1039">
-        <v>1038</v>
-      </c>
-      <c r="B1039" t="s">
-        <v>79</v>
-      </c>
-      <c r="C1039">
-        <v>10</v>
-      </c>
-      <c r="D1039" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1040" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1040">
-        <v>1039</v>
-      </c>
-      <c r="B1040" t="s">
-        <v>78</v>
-      </c>
-      <c r="C1040">
-        <v>10</v>
-      </c>
-      <c r="D1040" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1041" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1041">
-        <v>1040</v>
-      </c>
-      <c r="B1041" t="s">
-        <v>77</v>
-      </c>
-      <c r="C1041">
-        <v>10</v>
-      </c>
-      <c r="D1041" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1042" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1042">
-        <v>1041</v>
-      </c>
-      <c r="B1042" t="s">
-        <v>76</v>
-      </c>
-      <c r="C1042">
-        <v>6</v>
-      </c>
-      <c r="D1042" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1043" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1043">
-        <v>1042</v>
-      </c>
-      <c r="B1043" t="s">
-        <v>75</v>
-      </c>
-      <c r="C1043">
-        <v>6</v>
-      </c>
-      <c r="D1043" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1044" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1044">
-        <v>1043</v>
-      </c>
-      <c r="B1044" t="s">
-        <v>74</v>
-      </c>
-      <c r="C1044">
-        <v>40</v>
-      </c>
-      <c r="D1044" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1045" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1045">
-        <v>1044</v>
-      </c>
-      <c r="B1045" t="s">
-        <v>73</v>
-      </c>
-      <c r="C1045">
-        <v>4</v>
-      </c>
-      <c r="D1045" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1046" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1046">
-        <v>1045</v>
-      </c>
-      <c r="B1046" t="s">
-        <v>72</v>
-      </c>
-      <c r="C1046">
-        <v>1</v>
-      </c>
-      <c r="D1046" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1047" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1047">
-        <v>1046</v>
-      </c>
-      <c r="B1047" t="s">
-        <v>71</v>
-      </c>
-      <c r="C1047">
-        <v>4</v>
-      </c>
-      <c r="D1047" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1048" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1048">
-        <v>1047</v>
-      </c>
-      <c r="B1048" t="s">
-        <v>70</v>
-      </c>
-      <c r="C1048">
-        <v>4</v>
-      </c>
-      <c r="D1048" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1049" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1049">
-        <v>1048</v>
-      </c>
-      <c r="B1049" t="s">
-        <v>69</v>
-      </c>
-      <c r="C1049">
-        <v>4</v>
-      </c>
-      <c r="D1049" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1050" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1050">
-        <v>1049</v>
-      </c>
-      <c r="B1050" t="s">
-        <v>68</v>
-      </c>
-      <c r="C1050">
-        <v>1</v>
-      </c>
-      <c r="D1050" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1051" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1051">
-        <v>1050</v>
-      </c>
-      <c r="B1051" t="s">
-        <v>67</v>
-      </c>
-      <c r="C1051">
-        <v>60</v>
-      </c>
-      <c r="D1051" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1052" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1052">
-        <v>1051</v>
-      </c>
-      <c r="B1052" t="s">
-        <v>66</v>
-      </c>
-      <c r="C1052">
-        <v>60</v>
-      </c>
-      <c r="D1052" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1053" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1053">
-        <v>1052</v>
-      </c>
-      <c r="B1053" t="s">
-        <v>65</v>
-      </c>
-      <c r="C1053">
-        <v>60</v>
-      </c>
-      <c r="D1053" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1054" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1054">
-        <v>1053</v>
-      </c>
-      <c r="B1054" t="s">
-        <v>64</v>
-      </c>
-      <c r="C1054">
-        <v>60</v>
-      </c>
-      <c r="D1054" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1055" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1055">
-        <v>1054</v>
-      </c>
-      <c r="B1055" t="s">
-        <v>63</v>
-      </c>
-      <c r="C1055">
-        <v>60</v>
-      </c>
-      <c r="D1055" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1056" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1056">
-        <v>1055</v>
-      </c>
-      <c r="B1056" t="s">
-        <v>62</v>
-      </c>
-      <c r="C1056">
-        <v>60</v>
-      </c>
-      <c r="D1056" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1057" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1057">
-        <v>1056</v>
-      </c>
-      <c r="B1057" t="s">
-        <v>61</v>
-      </c>
-      <c r="C1057">
-        <v>60</v>
-      </c>
-      <c r="D1057" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1058" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1058">
-        <v>1057</v>
-      </c>
-      <c r="B1058" t="s">
-        <v>60</v>
-      </c>
-      <c r="C1058">
-        <v>30</v>
-      </c>
-      <c r="D1058" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1059" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1059">
-        <v>1058</v>
-      </c>
-      <c r="B1059" t="s">
-        <v>59</v>
-      </c>
-      <c r="C1059">
-        <v>40</v>
-      </c>
-      <c r="D1059" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1060" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1060">
-        <v>1059</v>
-      </c>
-      <c r="B1060" t="s">
-        <v>58</v>
-      </c>
-      <c r="C1060">
-        <v>63</v>
-      </c>
-      <c r="D1060" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1061" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1061">
-        <v>1060</v>
-      </c>
-      <c r="B1061" t="s">
-        <v>57</v>
-      </c>
-      <c r="C1061">
-        <v>10</v>
-      </c>
-      <c r="D1061" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1062" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1062">
-        <v>1061</v>
-      </c>
-      <c r="B1062" t="s">
-        <v>56</v>
-      </c>
-      <c r="C1062">
-        <v>40</v>
-      </c>
-      <c r="D1062" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1063" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1063">
-        <v>1062</v>
-      </c>
-      <c r="B1063" t="s">
-        <v>55</v>
-      </c>
-      <c r="C1063">
-        <v>60</v>
-      </c>
-      <c r="D1063" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1064" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1064">
-        <v>1063</v>
-      </c>
-      <c r="B1064" t="s">
-        <v>54</v>
-      </c>
-      <c r="C1064">
-        <v>6</v>
-      </c>
-      <c r="D1064" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1065" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1065">
-        <v>1064</v>
-      </c>
-      <c r="B1065" t="s">
-        <v>53</v>
-      </c>
-      <c r="C1065">
-        <v>18</v>
-      </c>
-      <c r="D1065" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1066" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1066">
-        <v>1065</v>
-      </c>
-      <c r="B1066" t="s">
-        <v>52</v>
-      </c>
-      <c r="C1066">
-        <v>8</v>
-      </c>
-      <c r="D1066" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1067" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1067">
-        <v>1066</v>
-      </c>
-      <c r="B1067" t="s">
-        <v>51</v>
-      </c>
-      <c r="C1067">
-        <v>30</v>
-      </c>
-      <c r="D1067" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1068" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1068">
-        <v>1067</v>
-      </c>
-      <c r="B1068" t="s">
-        <v>50</v>
-      </c>
-      <c r="C1068">
-        <v>2</v>
-      </c>
-      <c r="D1068" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1069" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1069">
-        <v>1068</v>
-      </c>
-      <c r="B1069" t="s">
-        <v>49</v>
-      </c>
-      <c r="C1069">
-        <v>5</v>
-      </c>
-      <c r="D1069" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1070" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1070">
-        <v>1069</v>
-      </c>
-      <c r="B1070" t="s">
-        <v>48</v>
-      </c>
-      <c r="C1070">
-        <v>5</v>
-      </c>
-      <c r="D1070" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1071" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1071">
-        <v>1070</v>
-      </c>
-      <c r="B1071" t="s">
-        <v>47</v>
-      </c>
-      <c r="C1071">
-        <v>5</v>
-      </c>
-      <c r="D1071" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1072" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1072">
-        <v>1071</v>
-      </c>
-      <c r="B1072" t="s">
-        <v>46</v>
-      </c>
-      <c r="C1072">
-        <v>5</v>
-      </c>
-      <c r="D1072" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1073" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1073">
-        <v>1072</v>
-      </c>
-      <c r="B1073" t="s">
-        <v>45</v>
-      </c>
-      <c r="C1073">
-        <v>20</v>
-      </c>
-      <c r="D1073" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1074" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1074">
-        <v>1073</v>
-      </c>
-      <c r="B1074" t="s">
-        <v>44</v>
-      </c>
-      <c r="C1074">
-        <v>240</v>
-      </c>
-      <c r="D1074" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1075" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1075">
-        <v>1074</v>
-      </c>
-      <c r="B1075" t="s">
-        <v>43</v>
-      </c>
-      <c r="C1075">
-        <v>120</v>
-      </c>
-      <c r="D1075" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1076" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1076">
-        <v>1075</v>
-      </c>
-      <c r="B1076" t="s">
-        <v>42</v>
-      </c>
-      <c r="C1076">
-        <v>60</v>
-      </c>
-      <c r="D1076" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1077" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1077">
-        <v>1076</v>
-      </c>
-      <c r="B1077" t="s">
-        <v>41</v>
-      </c>
-      <c r="C1077">
-        <v>120</v>
-      </c>
-      <c r="D1077" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1078" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1078">
-        <v>1077</v>
-      </c>
-      <c r="B1078" t="s">
-        <v>40</v>
-      </c>
-      <c r="C1078">
-        <v>72</v>
-      </c>
-      <c r="D1078" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1079" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1079">
-        <v>1078</v>
-      </c>
-      <c r="B1079" t="s">
-        <v>39</v>
-      </c>
-      <c r="C1079">
-        <v>60</v>
-      </c>
-      <c r="D1079" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1080" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1080">
-        <v>1079</v>
-      </c>
-      <c r="B1080" t="s">
-        <v>38</v>
-      </c>
-      <c r="C1080">
-        <v>120</v>
-      </c>
-      <c r="D1080" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1081" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1081">
-        <v>1080</v>
-      </c>
-      <c r="B1081" t="s">
-        <v>37</v>
-      </c>
-      <c r="C1081">
-        <v>72</v>
-      </c>
-      <c r="D1081" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1082" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1082">
-        <v>1081</v>
-      </c>
-      <c r="B1082" t="s">
-        <v>36</v>
-      </c>
-      <c r="C1082">
-        <v>20</v>
-      </c>
-      <c r="D1082" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1083" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1083">
-        <v>1082</v>
-      </c>
-      <c r="B1083" t="s">
-        <v>35</v>
-      </c>
-      <c r="C1083">
-        <v>100</v>
-      </c>
-      <c r="D1083" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1084" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1084">
-        <v>1083</v>
-      </c>
-      <c r="B1084" t="s">
-        <v>34</v>
-      </c>
-      <c r="C1084">
-        <v>5</v>
-      </c>
-      <c r="D1084" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1085" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1085">
-        <v>1084</v>
-      </c>
-      <c r="B1085" t="s">
-        <v>33</v>
-      </c>
-      <c r="C1085">
-        <v>10</v>
-      </c>
-      <c r="D1085" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1086" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1086">
-        <v>1085</v>
-      </c>
-      <c r="B1086" t="s">
-        <v>32</v>
-      </c>
-      <c r="C1086">
-        <v>20</v>
-      </c>
-      <c r="D1086" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1087" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1087">
-        <v>1086</v>
-      </c>
-      <c r="B1087" t="s">
-        <v>31</v>
-      </c>
-      <c r="C1087">
-        <v>20</v>
-      </c>
-      <c r="D1087" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1088" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1088">
-        <v>1087</v>
-      </c>
-      <c r="B1088" t="s">
-        <v>30</v>
-      </c>
-      <c r="C1088">
-        <v>24</v>
-      </c>
-      <c r="D1088" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1089" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1089">
-        <v>1088</v>
-      </c>
-      <c r="B1089" t="s">
-        <v>29</v>
-      </c>
-      <c r="C1089">
-        <v>240</v>
-      </c>
-      <c r="D1089" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1090" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1090">
-        <v>1089</v>
-      </c>
-      <c r="B1090" t="s">
-        <v>28</v>
-      </c>
-      <c r="C1090">
-        <v>240</v>
-      </c>
-      <c r="D1090" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1091" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1091">
-        <v>1090</v>
-      </c>
-      <c r="B1091" t="s">
-        <v>27</v>
-      </c>
-      <c r="C1091">
-        <v>480</v>
-      </c>
-      <c r="D1091" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1092" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1092">
-        <v>1091</v>
-      </c>
-      <c r="B1092" t="s">
-        <v>26</v>
-      </c>
-      <c r="C1092">
-        <v>120</v>
-      </c>
-      <c r="D1092" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1093" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1093">
-        <v>1092</v>
-      </c>
-      <c r="B1093" t="s">
-        <v>25</v>
-      </c>
-      <c r="C1093">
-        <v>240</v>
-      </c>
-      <c r="D1093" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1094" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1094">
-        <v>1093</v>
-      </c>
-      <c r="B1094" t="s">
-        <v>24</v>
-      </c>
-      <c r="C1094">
-        <v>240</v>
-      </c>
-      <c r="D1094" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1095" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1095">
-        <v>1094</v>
-      </c>
-      <c r="B1095" t="s">
-        <v>23</v>
-      </c>
-      <c r="C1095">
-        <v>480</v>
-      </c>
-      <c r="D1095" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1096" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1096">
-        <v>1095</v>
-      </c>
-      <c r="B1096" t="s">
-        <v>22</v>
-      </c>
-      <c r="C1096">
-        <v>120</v>
-      </c>
-      <c r="D1096" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1097" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1097">
-        <v>1096</v>
-      </c>
-      <c r="B1097" t="s">
-        <v>21</v>
-      </c>
-      <c r="C1097">
-        <v>120</v>
-      </c>
-      <c r="D1097" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1098" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1098">
-        <v>1097</v>
-      </c>
-      <c r="B1098" t="s">
-        <v>20</v>
-      </c>
-      <c r="C1098">
-        <v>120</v>
-      </c>
-      <c r="D1098" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1099" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1099">
-        <v>1098</v>
-      </c>
-      <c r="B1099" t="s">
-        <v>19</v>
-      </c>
-      <c r="C1099">
-        <v>12</v>
-      </c>
-      <c r="D1099" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1100" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1100">
-        <v>1099</v>
-      </c>
-      <c r="B1100" t="s">
-        <v>18</v>
-      </c>
-      <c r="C1100">
-        <v>12</v>
-      </c>
-      <c r="D1100" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1101" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1101">
-        <v>1100</v>
-      </c>
-      <c r="B1101" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1101">
-        <v>30</v>
-      </c>
-      <c r="D1101" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1102" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1102">
-        <v>1101</v>
-      </c>
-      <c r="B1102" t="s">
-        <v>16</v>
-      </c>
-      <c r="C1102">
-        <v>12</v>
-      </c>
-      <c r="D1102" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1103" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1103">
-        <v>1102</v>
-      </c>
-      <c r="B1103" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1103">
-        <v>6</v>
-      </c>
-      <c r="D1103" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1104" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1104">
-        <v>1103</v>
-      </c>
-      <c r="B1104" t="s">
-        <v>14</v>
-      </c>
-      <c r="C1104">
-        <v>1</v>
-      </c>
-      <c r="D1104" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1105" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1105">
-        <v>1104</v>
-      </c>
-      <c r="B1105" t="s">
-        <v>13</v>
-      </c>
-      <c r="C1105">
-        <v>20</v>
-      </c>
-      <c r="D1105" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1106" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1106">
-        <v>1105</v>
-      </c>
-      <c r="B1106" t="s">
-        <v>12</v>
-      </c>
-      <c r="C1106">
-        <v>20</v>
-      </c>
-      <c r="D1106" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1107" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1107">
-        <v>1106</v>
-      </c>
-      <c r="B1107" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1107">
-        <v>20</v>
-      </c>
-      <c r="D1107" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1108" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1108">
-        <v>1107</v>
-      </c>
-      <c r="B1108" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1108">
-        <v>56</v>
-      </c>
-      <c r="D1108" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1109" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1109">
-        <v>1108</v>
-      </c>
-      <c r="B1109" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1109">
-        <v>50</v>
-      </c>
-      <c r="D1109" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1110" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1110">
-        <v>1109</v>
-      </c>
-      <c r="B1110" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1110">
-        <v>50</v>
-      </c>
-      <c r="D1110" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1111" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1111">
-        <v>1110</v>
-      </c>
-      <c r="B1111" t="s">
-        <v>7</v>
-      </c>
-      <c r="C1111">
-        <v>50</v>
-      </c>
-      <c r="D1111" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1112" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1112">
-        <v>1111</v>
-      </c>
-      <c r="B1112" t="s">
-        <v>6</v>
-      </c>
-      <c r="C1112">
-        <v>50</v>
-      </c>
-      <c r="D1112" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1113" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1113">
-        <v>1112</v>
-      </c>
-      <c r="B1113" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1113">
-        <v>50</v>
-      </c>
-      <c r="D1113" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1114" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1114">
-        <v>1113</v>
-      </c>
-      <c r="B1114" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1114">
-        <v>50</v>
-      </c>
-      <c r="D1114" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1115" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1115">
-        <v>1114</v>
-      </c>
-      <c r="B1115" t="s">
-        <v>3</v>
-      </c>
-      <c r="C1115">
-        <v>100</v>
-      </c>
-      <c r="D1115" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1116" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1116">
-        <v>1115</v>
-      </c>
-      <c r="B1116" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1116">
-        <v>60</v>
-      </c>
-      <c r="D1116" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1117" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1117">
-        <v>1116</v>
-      </c>
-      <c r="B1117" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1117">
-        <v>100</v>
-      </c>
-      <c r="D1117" t="s">
-        <v>968</v>
-      </c>
-    </row>
-    <row r="1118" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1118">
-        <v>1117</v>
-      </c>
-      <c r="B1118" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1118">
-        <v>80</v>
-      </c>
-      <c r="D1118" t="s">
-        <v>968</v>
+        <v>967</v>
       </c>
     </row>
   </sheetData>

</xml_diff>